<commit_message>
Fix Midi Note 0
Also added another Bb fingering
Added research into trills.
</commit_message>
<xml_diff>
--- a/Sax_Fingering_details.xlsx
+++ b/Sax_Fingering_details.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tim\Documents\GitHub\MIDI-Wind-Controller\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF89A73-932C-446F-B66A-EF2E7B01359E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAFCB408-2611-49EF-9B1D-09867BB74FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29355" yWindow="240" windowWidth="26775" windowHeight="16260" activeTab="2" xr2:uid="{37DECD7E-2A26-408F-B389-C3EB14E31A56}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="2" xr2:uid="{37DECD7E-2A26-408F-B389-C3EB14E31A56}"/>
   </bookViews>
   <sheets>
     <sheet name="Leonardo" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="88">
   <si>
     <t>C#</t>
   </si>
@@ -6416,7 +6416,7 @@
       <c r="T15" s="1"/>
       <c r="U15" s="1"/>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>77</v>
       </c>
@@ -6430,7 +6430,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>73</v>
       </c>
@@ -6441,7 +6441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>75</v>
       </c>
@@ -6454,7 +6454,7 @@
       <c r="F20" s="4"/>
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B21">
         <f>B19+B20*2</f>
         <v>2</v>
@@ -6470,30 +6470,30 @@
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
     </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
     </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>76</v>
       </c>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>78</v>
       </c>
       <c r="G25" t="s">
         <v>80</v>
       </c>
-      <c r="R25" s="7" t="s">
+      <c r="S25" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="S25" s="7"/>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T25" s="7"/>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>79</v>
       </c>
@@ -6523,31 +6523,34 @@
         <v>46</v>
       </c>
       <c r="L26" s="1">
+        <v>46</v>
+      </c>
+      <c r="M26" s="1">
         <v>45</v>
       </c>
-      <c r="M26" s="1">
+      <c r="N26" s="1">
         <v>42</v>
       </c>
-      <c r="N26" s="1">
+      <c r="O26" s="1">
         <v>41</v>
       </c>
-      <c r="O26" s="1">
+      <c r="P26" s="1">
         <v>40</v>
       </c>
-      <c r="P26" s="1">
+      <c r="Q26" s="1">
         <v>39</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="R26" s="1">
         <v>38</v>
       </c>
-      <c r="R26" s="1">
+      <c r="S26" s="1">
         <v>37</v>
       </c>
-      <c r="S26" s="1">
+      <c r="T26" s="1">
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>13</v>
       </c>
@@ -6580,31 +6583,34 @@
         <v>4</v>
       </c>
       <c r="L27" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="M27" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="M27" s="1" t="s">
+      <c r="N27" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="N27" s="1" t="s">
+      <c r="O27" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="O27" s="1" t="s">
+      <c r="P27" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="P27" s="1" t="s">
+      <c r="Q27" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="Q27" s="1" t="s">
+      <c r="R27" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="R27" s="1" t="s">
-        <v>0</v>
-      </c>
       <c r="S27" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="T27" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>74</v>
       </c>
@@ -6619,7 +6625,6 @@
       <c r="H28" s="2"/>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
-      <c r="L28" s="3"/>
       <c r="M28" s="3"/>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
@@ -6627,8 +6632,9 @@
       <c r="Q28" s="3"/>
       <c r="R28" s="3"/>
       <c r="S28" s="3"/>
-    </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T28" s="3"/>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>2</v>
       </c>
@@ -6655,7 +6661,7 @@
       <c r="K29" s="2">
         <v>1</v>
       </c>
-      <c r="L29" s="3">
+      <c r="L29" s="2">
         <v>1</v>
       </c>
       <c r="M29" s="3">
@@ -6679,8 +6685,11 @@
       <c r="S29" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T29" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>3</v>
       </c>
@@ -6703,7 +6712,7 @@
       <c r="L30" s="2">
         <v>1</v>
       </c>
-      <c r="M30" s="3">
+      <c r="M30" s="2">
         <v>1</v>
       </c>
       <c r="N30" s="3">
@@ -6724,8 +6733,11 @@
       <c r="S30" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T30" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>6</v>
       </c>
@@ -6738,10 +6750,7 @@
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="2">
-        <v>1</v>
-      </c>
+      <c r="M31" s="2"/>
       <c r="N31" s="2">
         <v>1</v>
       </c>
@@ -6760,8 +6769,11 @@
       <c r="S31" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T31" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>72</v>
       </c>
@@ -6789,7 +6801,7 @@
       <c r="M32" s="2">
         <v>1</v>
       </c>
-      <c r="N32" s="3">
+      <c r="N32" s="2">
         <v>1</v>
       </c>
       <c r="O32" s="3">
@@ -6807,8 +6819,11 @@
       <c r="S32" s="3">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T32" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>71</v>
       </c>
@@ -6821,16 +6836,16 @@
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
-      <c r="L33" s="2"/>
-      <c r="M33" s="3"/>
-      <c r="N33" s="2"/>
-      <c r="O33" s="3"/>
+      <c r="M33" s="2"/>
+      <c r="N33" s="3"/>
+      <c r="O33" s="2"/>
       <c r="P33" s="3"/>
       <c r="Q33" s="3"/>
       <c r="R33" s="3"/>
       <c r="S33" s="3"/>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T33" s="3"/>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>24</v>
       </c>
@@ -6854,12 +6869,13 @@
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
-      <c r="P34" s="3"/>
+      <c r="P34" s="2"/>
       <c r="Q34" s="3"/>
       <c r="R34" s="3"/>
       <c r="S34" s="3"/>
-    </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T34" s="3"/>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>7</v>
       </c>
@@ -6877,18 +6893,18 @@
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
-      <c r="L35" s="2"/>
+      <c r="L35">
+        <v>1</v>
+      </c>
       <c r="M35" s="2"/>
-      <c r="N35" s="2">
-        <v>1</v>
-      </c>
+      <c r="N35" s="2"/>
       <c r="O35" s="2">
         <v>1</v>
       </c>
-      <c r="P35" s="3">
-        <v>1</v>
-      </c>
-      <c r="Q35" s="2">
+      <c r="P35" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q35" s="3">
         <v>1</v>
       </c>
       <c r="R35" s="2">
@@ -6897,8 +6913,11 @@
       <c r="S35" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T35" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>9</v>
       </c>
@@ -6911,18 +6930,15 @@
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
-      <c r="L36" s="2"/>
-      <c r="M36" s="2">
-        <v>1</v>
-      </c>
-      <c r="N36" s="2"/>
-      <c r="O36" s="2">
-        <v>1</v>
-      </c>
-      <c r="P36" s="3">
-        <v>1</v>
-      </c>
-      <c r="Q36" s="2">
+      <c r="M36" s="2"/>
+      <c r="N36" s="2">
+        <v>1</v>
+      </c>
+      <c r="O36" s="2"/>
+      <c r="P36" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q36" s="3">
         <v>1</v>
       </c>
       <c r="R36" s="2">
@@ -6931,8 +6947,11 @@
       <c r="S36" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T36" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>11</v>
       </c>
@@ -6945,14 +6964,11 @@
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
-      <c r="L37" s="2"/>
       <c r="M37" s="2"/>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
-      <c r="P37" s="3">
-        <v>1</v>
-      </c>
-      <c r="Q37" s="2">
+      <c r="P37" s="2"/>
+      <c r="Q37" s="3">
         <v>1</v>
       </c>
       <c r="R37" s="2">
@@ -6961,8 +6977,11 @@
       <c r="S37" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T37" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>68</v>
       </c>
@@ -6975,18 +6994,18 @@
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
-      <c r="L38" s="2"/>
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
-      <c r="P38" s="3">
-        <v>1</v>
-      </c>
-      <c r="Q38" s="2"/>
+      <c r="P38" s="2"/>
+      <c r="Q38" s="3">
+        <v>1</v>
+      </c>
       <c r="R38" s="2"/>
       <c r="S38" s="2"/>
-    </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T38" s="2"/>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>1</v>
       </c>
@@ -6996,20 +7015,20 @@
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
-      <c r="L39" s="2"/>
       <c r="M39" s="2"/>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
-      <c r="P39" s="3"/>
-      <c r="Q39" s="2"/>
-      <c r="R39" s="2">
-        <v>1</v>
-      </c>
+      <c r="P39" s="2"/>
+      <c r="Q39" s="3"/>
+      <c r="R39" s="2"/>
       <c r="S39" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T39" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>81</v>
       </c>
@@ -7034,7 +7053,7 @@
         <v>16</v>
       </c>
       <c r="H40" s="1">
-        <f t="shared" ref="H40:K40" si="2">H28*1+H29*2+H30*4+H31*8+H32*16+H33*32+H34*64+H35*128+H36*256+H37*512+H38*1024+H39*2048</f>
+        <f t="shared" ref="H40:L40" si="2">H28*1+H29*2+H30*4+H31*8+H32*16+H33*32+H34*64+H35*128+H36*256+H37*512+H38*1024+H39*2048</f>
         <v>20</v>
       </c>
       <c r="I40" s="1">
@@ -7050,42 +7069,46 @@
         <v>82</v>
       </c>
       <c r="L40" s="1">
-        <f t="shared" ref="L40:S40" si="3">L28*1+L29*2+L30*4+L31*8+L32*16+L33*32+L34*64+L35*128+L36*256+L37*512+L38*1024+L39*2048</f>
+        <f t="shared" si="2"/>
+        <v>150</v>
+      </c>
+      <c r="M40" s="1">
+        <f t="shared" ref="M40:T40" si="3">M28*1+M29*2+M30*4+M31*8+M32*16+M33*32+M34*64+M35*128+M36*256+M37*512+M38*1024+M39*2048</f>
         <v>22</v>
       </c>
-      <c r="M40" s="1">
+      <c r="N40" s="1">
         <f t="shared" si="3"/>
         <v>286</v>
       </c>
-      <c r="N40" s="1">
+      <c r="O40" s="1">
         <f t="shared" si="3"/>
         <v>158</v>
       </c>
-      <c r="O40" s="1">
+      <c r="P40" s="1">
         <f t="shared" si="3"/>
         <v>414</v>
       </c>
-      <c r="P40" s="1">
+      <c r="Q40" s="1">
         <f t="shared" si="3"/>
         <v>1950</v>
       </c>
-      <c r="Q40" s="1">
+      <c r="R40" s="1">
         <f t="shared" si="3"/>
         <v>926</v>
-      </c>
-      <c r="R40" s="1">
-        <f t="shared" si="3"/>
-        <v>2974</v>
       </c>
       <c r="S40" s="1">
         <f t="shared" si="3"/>
         <v>2974</v>
       </c>
-    </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T40" s="1">
+        <f t="shared" si="3"/>
+        <v>2974</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>61</v>
       </c>
@@ -7093,7 +7116,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>13</v>
       </c>
@@ -7128,7 +7151,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>74</v>
       </c>
@@ -7163,7 +7186,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>2</v>
       </c>
@@ -7198,7 +7221,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>3</v>
       </c>
@@ -7231,7 +7254,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>6</v>
       </c>
@@ -7266,7 +7289,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>72</v>
       </c>
@@ -7645,7 +7668,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B28:C39 E28:E39 G28:J39 L28:S39 K29 K32">
+  <conditionalFormatting sqref="B28:C39 E28:E39 G28:J39 M28:T39 K29:L29 L30 K32:L32 L34">
     <cfRule type="cellIs" dxfId="7" priority="7" operator="lessThan">
       <formula>1</formula>
     </cfRule>
@@ -7669,7 +7692,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G44:I58 K47:K58 L47:L55 K44:L45">
+  <conditionalFormatting sqref="K44:L45 G44:I58 L47:L55 K47:K58">
     <cfRule type="cellIs" dxfId="1" priority="5" operator="lessThan">
       <formula>1</formula>
     </cfRule>

</xml_diff>